<commit_message>
Created excel, csv and script for analysing Lissorhoptrus abundance from salabra data
</commit_message>
<xml_diff>
--- a/data/original/Birds.xlsx
+++ b/data/original/Birds.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://irtacat-my.sharepoint.com/personal/alejandro_munoz_irta_cat/Documents/Documentos/Exclusion-Lisso-Analysis/data/original/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51580A9F-30DF-4995-84A3-25A12842FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{51580A9F-30DF-4995-84A3-25A12842FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE4C42B4-7501-4ED6-91CB-6BD4A124E714}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4F6AF7F5-EA7B-447A-A017-3996FC650096}"/>
   </bookViews>
@@ -214,6 +214,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Continue working on the lisso abundance screening script. Created script for lisso abundance models.
</commit_message>
<xml_diff>
--- a/data/original/Birds.xlsx
+++ b/data/original/Birds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://irtacat-my.sharepoint.com/personal/alejandro_munoz_irta_cat/Documents/Documentos/Exclusion-Lisso-Analysis/data/original/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{51580A9F-30DF-4995-84A3-25A12842FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE4C42B4-7501-4ED6-91CB-6BD4A124E714}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{51580A9F-30DF-4995-84A3-25A12842FA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32E07C98-EC82-42FA-8487-F5A6AA1549EB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4F6AF7F5-EA7B-447A-A017-3996FC650096}"/>
   </bookViews>
@@ -214,10 +214,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -537,6 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B62120D8-0F9B-412D-881D-577439C2240E}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -566,7 +563,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -589,7 +586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -612,7 +609,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -635,7 +632,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -658,7 +655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -681,7 +678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -704,7 +701,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
@@ -727,7 +724,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
@@ -750,7 +747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -773,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
@@ -796,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
@@ -819,7 +816,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
@@ -842,7 +839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1</v>
       </c>
@@ -865,7 +862,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1</v>
       </c>
@@ -888,7 +885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1</v>
       </c>
@@ -934,7 +931,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1</v>
       </c>
@@ -957,7 +954,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2</v>
       </c>
@@ -980,7 +977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2</v>
       </c>
@@ -1003,7 +1000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2</v>
       </c>
@@ -1026,7 +1023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2</v>
       </c>
@@ -1049,7 +1046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2</v>
       </c>
@@ -1072,7 +1069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2</v>
       </c>
@@ -1095,7 +1092,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2</v>
       </c>
@@ -1118,7 +1115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2</v>
       </c>
@@ -1141,7 +1138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2</v>
       </c>
@@ -1164,7 +1161,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2</v>
       </c>
@@ -1187,7 +1184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2</v>
       </c>
@@ -1210,7 +1207,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2</v>
       </c>
@@ -1233,7 +1230,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2</v>
       </c>
@@ -1256,7 +1253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2</v>
       </c>
@@ -1279,7 +1276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2</v>
       </c>
@@ -1325,7 +1322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1348,7 +1345,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3</v>
       </c>
@@ -1371,7 +1368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>3</v>
       </c>
@@ -1394,7 +1391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>3</v>
       </c>
@@ -1417,7 +1414,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>3</v>
       </c>
@@ -1440,7 +1437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>3</v>
       </c>
@@ -1463,7 +1460,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>3</v>
       </c>
@@ -1486,7 +1483,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>3</v>
       </c>
@@ -1509,7 +1506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>3</v>
       </c>
@@ -1532,7 +1529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>3</v>
       </c>
@@ -1555,7 +1552,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>3</v>
       </c>
@@ -1578,7 +1575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>3</v>
       </c>
@@ -1601,7 +1598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>3</v>
       </c>
@@ -1624,7 +1621,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>3</v>
       </c>
@@ -1647,7 +1644,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1670,7 +1667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>3</v>
       </c>
@@ -1716,7 +1713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>3</v>
       </c>
@@ -1739,7 +1736,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>4</v>
       </c>
@@ -1762,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>4</v>
       </c>
@@ -1785,7 +1782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>4</v>
       </c>
@@ -1808,7 +1805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>4</v>
       </c>
@@ -1831,7 +1828,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>4</v>
       </c>
@@ -1854,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>4</v>
       </c>
@@ -1877,7 +1874,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>4</v>
       </c>
@@ -1900,7 +1897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>4</v>
       </c>
@@ -1923,7 +1920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>4</v>
       </c>
@@ -1946,7 +1943,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>4</v>
       </c>
@@ -1969,7 +1966,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>4</v>
       </c>
@@ -1992,7 +1989,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>4</v>
       </c>
@@ -2015,7 +2012,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>4</v>
       </c>
@@ -2038,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>4</v>
       </c>
@@ -2061,7 +2058,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>4</v>
       </c>
@@ -2107,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>4</v>
       </c>
@@ -2130,7 +2127,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>5</v>
       </c>
@@ -2153,7 +2150,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>5</v>
       </c>
@@ -2176,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>5</v>
       </c>
@@ -2199,7 +2196,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>5</v>
       </c>
@@ -2222,7 +2219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>5</v>
       </c>
@@ -2245,7 +2242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>5</v>
       </c>
@@ -2268,7 +2265,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>5</v>
       </c>
@@ -2291,7 +2288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>5</v>
       </c>
@@ -2314,7 +2311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>5</v>
       </c>
@@ -2337,7 +2334,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>5</v>
       </c>
@@ -2360,7 +2357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>5</v>
       </c>
@@ -2383,7 +2380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>5</v>
       </c>
@@ -2406,7 +2403,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>5</v>
       </c>
@@ -2429,7 +2426,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>5</v>
       </c>
@@ -2452,7 +2449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>5</v>
       </c>
@@ -2498,7 +2495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>5</v>
       </c>
@@ -2521,7 +2518,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>36</v>
       </c>
@@ -2544,7 +2541,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>36</v>
       </c>
@@ -2567,7 +2564,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>36</v>
       </c>
@@ -2590,7 +2587,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>36</v>
       </c>
@@ -2613,7 +2610,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>36</v>
       </c>
@@ -2636,7 +2633,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>36</v>
       </c>
@@ -2659,7 +2656,7 @@
         <v>56.8</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>36</v>
       </c>
@@ -2682,7 +2679,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>36</v>
       </c>
@@ -2705,7 +2702,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>36</v>
       </c>
@@ -2728,7 +2725,7 @@
         <v>24.8</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>36</v>
       </c>
@@ -2751,7 +2748,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>36</v>
       </c>
@@ -2774,7 +2771,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>36</v>
       </c>
@@ -2797,7 +2794,7 @@
         <v>7.6</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>36</v>
       </c>
@@ -2820,7 +2817,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>36</v>
       </c>
@@ -2843,7 +2840,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>36</v>
       </c>
@@ -2889,7 +2886,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>36</v>
       </c>
@@ -2913,7 +2910,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G103" xr:uid="{0C67C03B-E7D6-46D0-812A-5B13F3D88FE4}"/>
+  <autoFilter ref="A1:G103" xr:uid="{0C67C03B-E7D6-46D0-812A-5B13F3D88FE4}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Sturnus"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>